<commit_message>
Story: crown jewels in oval and rose cuts (owner)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sispid5Qo8kvdYnx3crKZR
</commit_message>
<xml_diff>
--- a/docs/SpriteChecklist.xlsx
+++ b/docs/SpriteChecklist.xlsx
@@ -47300,7 +47300,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Pear Emerald</t>
+          <t>Rose Emerald</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -47319,7 +47319,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Pear Sapphire</t>
+          <t>Rose Sapphire</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -47338,7 +47338,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Pear Ruby</t>
+          <t>Rose Ruby</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">

</xml_diff>